<commit_message>
Manage Email/Text to Pay +ve cases
</commit_message>
<xml_diff>
--- a/KatalonData/EmailTextToPay/ManualEntry_Prod.xlsx
+++ b/KatalonData/EmailTextToPay/ManualEntry_Prod.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t470258\Documents\VPS-Katalon\KatalonData\EmailTextToPay\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78CDF8F8-B02F-4DF6-A538-F2D7646005D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr documentId="13_ncr:1_{78CDF8F8-B02F-4DF6-A538-F2D7646005D7}" revIDLastSave="0" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{A171AD99-6CB3-481A-968B-971B4AF2105E}"/>
+    <workbookView activeTab="1" windowHeight="11500" windowWidth="19420" xWindow="-110" xr2:uid="{A171AD99-6CB3-481A-968B-971B4AF2105E}" yWindow="-110"/>
   </bookViews>
   <sheets>
-    <sheet name="ManualEntry" sheetId="1" r:id="rId1"/>
-    <sheet name="ManualEntryError" sheetId="2" r:id="rId2"/>
+    <sheet name="ManualEntry" r:id="rId1" sheetId="1"/>
+    <sheet name="ManualEntryError" r:id="rId2" sheetId="2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="86">
   <si>
     <t>Result</t>
   </si>
@@ -289,12 +289,19 @@
   </si>
   <si>
     <t>Wed Mar 25 15:37:37 IST 2026</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Wed Apr 01 18:13:38 IST 2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -409,81 +416,81 @@
     </border>
   </borders>
   <cellStyleXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
+    <xf applyAlignment="0" applyBorder="0" applyFill="0" applyNumberFormat="0" applyProtection="0" borderId="0" fillId="0" fontId="4" numFmtId="0"/>
   </cellStyleXfs>
   <cellXfs count="22">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1" borderId="1" fillId="0" fontId="3" numFmtId="49" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf applyAlignment="1" applyFont="1" borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf applyAlignment="1" applyFont="1" borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+    <xf applyAlignment="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="4" numFmtId="49" xfId="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf applyAlignment="1" applyFont="1" applyNumberFormat="1" borderId="0" fillId="0" fontId="3" numFmtId="49" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf applyAlignment="1" applyFont="1" borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf applyAlignment="1" applyFont="1" borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1" borderId="1" fillId="0" fontId="3" numFmtId="49" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" borderId="2" fillId="2" fontId="3" numFmtId="49" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" borderId="2" fillId="3" fontId="3" numFmtId="49" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" borderId="1" fillId="3" fontId="3" numFmtId="49" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1" borderId="1" fillId="2" fontId="3" numFmtId="49" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1" borderId="1" fillId="0" fontId="5" numFmtId="49" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf applyAlignment="1" applyFont="1" borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf applyAlignment="1" applyFont="1" borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf applyAlignment="1" applyFont="1" borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle builtinId="8" name="Hyperlink" xfId="1"/>
+    <cellStyle builtinId="0" name="Normal" xfId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -500,10 +507,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -538,7 +545,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin panose="02110004020202020204" typeface="Aptos Display"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -590,7 +597,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin panose="02110004020202020204" typeface="Aptos Narrow"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -701,21 +708,21 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cap="flat" cmpd="sng" w="12700">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cap="flat" cmpd="sng" w="19050">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cap="flat" cmpd="sng" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -732,7 +739,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw algn="ctr" blurRad="57150" dir="5400000" dist="19050" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -804,42 +811,42 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" name="Office Theme" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F033DD18-DD0F-43E3-A2D0-6223D1731E2C}">
-  <dimension ref="A1:AA10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F033DD18-DD0F-43E3-A2D0-6223D1731E2C}">
+  <dimension ref="A1:AB10"/>
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.26953125" style="1" customWidth="1" collapsed="1"/>
-    <col min="2" max="2" width="15.36328125" style="19" customWidth="1" collapsed="1"/>
-    <col min="3" max="3" width="31.26953125" style="4" customWidth="1" collapsed="1"/>
-    <col min="4" max="4" width="8.08984375" style="1" customWidth="1" collapsed="1"/>
-    <col min="5" max="5" width="25.1796875" style="1" bestFit="1" customWidth="1" collapsed="1"/>
-    <col min="6" max="6" width="5.81640625" style="6" customWidth="1" collapsed="1"/>
-    <col min="7" max="7" width="8.1796875" style="6" customWidth="1" collapsed="1"/>
-    <col min="8" max="9" width="10.36328125" style="6" customWidth="1" collapsed="1"/>
-    <col min="10" max="10" width="17.7265625" style="6" customWidth="1" collapsed="1"/>
-    <col min="11" max="11" width="11.90625" style="6" customWidth="1" collapsed="1"/>
-    <col min="12" max="12" width="15" style="6" customWidth="1" collapsed="1"/>
-    <col min="13" max="14" width="14.453125" style="6" customWidth="1" collapsed="1"/>
-    <col min="15" max="15" width="7.81640625" style="6" customWidth="1" collapsed="1"/>
-    <col min="16" max="16" width="9.1796875" style="6" customWidth="1" collapsed="1"/>
-    <col min="17" max="17" width="13.90625" style="6" bestFit="1" customWidth="1" collapsed="1"/>
-    <col min="18" max="18" width="10.6328125" style="6" customWidth="1" collapsed="1"/>
-    <col min="19" max="19" width="10.81640625" style="6" bestFit="1" customWidth="1" collapsed="1"/>
-    <col min="20" max="20" width="8.1796875" style="6" customWidth="1" collapsed="1"/>
-    <col min="21" max="21" width="13.6328125" style="6" customWidth="1" collapsed="1"/>
-    <col min="22" max="22" width="15.453125" style="6" customWidth="1" collapsed="1"/>
-    <col min="23" max="27" width="8.7265625" style="6" collapsed="1"/>
-    <col min="28" max="16384" width="8.7265625" style="1" collapsed="1"/>
+    <col min="1" max="1" customWidth="true" style="1" width="6.26953125" collapsed="true"/>
+    <col min="2" max="2" customWidth="true" style="19" width="15.36328125" collapsed="true"/>
+    <col min="3" max="3" customWidth="true" style="4" width="31.26953125" collapsed="true"/>
+    <col min="4" max="4" customWidth="true" style="1" width="8.08984375" collapsed="true"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="1" width="25.1796875" collapsed="true"/>
+    <col min="6" max="6" customWidth="true" style="6" width="5.81640625" collapsed="true"/>
+    <col min="7" max="7" customWidth="true" style="6" width="8.1796875" collapsed="true"/>
+    <col min="8" max="9" customWidth="true" style="6" width="10.36328125" collapsed="true"/>
+    <col min="10" max="10" customWidth="true" style="6" width="17.7265625" collapsed="true"/>
+    <col min="11" max="11" customWidth="true" style="6" width="11.90625" collapsed="true"/>
+    <col min="12" max="12" customWidth="true" style="6" width="15.0" collapsed="true"/>
+    <col min="13" max="14" customWidth="true" style="6" width="14.453125" collapsed="true"/>
+    <col min="15" max="15" customWidth="true" style="6" width="7.81640625" collapsed="true"/>
+    <col min="16" max="16" customWidth="true" style="6" width="9.1796875" collapsed="true"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="6" width="13.90625" collapsed="true"/>
+    <col min="18" max="18" customWidth="true" style="6" width="10.6328125" collapsed="true"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="6" width="10.81640625" collapsed="true"/>
+    <col min="20" max="20" customWidth="true" style="6" width="8.1796875" collapsed="true"/>
+    <col min="21" max="21" customWidth="true" style="6" width="13.6328125" collapsed="true"/>
+    <col min="22" max="22" customWidth="true" style="6" width="15.453125" collapsed="true"/>
+    <col min="23" max="27" style="6" width="8.7265625" collapsed="true"/>
+    <col min="28" max="16384" style="1" width="8.7265625" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" s="3" customFormat="1" ht="25" x14ac:dyDescent="0.25">
+    <row customFormat="1" ht="25" r="1" s="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -922,7 +929,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:27" s="3" customFormat="1" ht="19" customHeight="1" x14ac:dyDescent="0.25">
+    <row customFormat="1" customHeight="1" ht="19" r="2" s="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>53</v>
       </c>
@@ -967,7 +974,7 @@
       <c r="Z2" s="9"/>
       <c r="AA2" s="9"/>
     </row>
-    <row r="3" spans="1:27" ht="21.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row customHeight="1" ht="21.5" r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>53</v>
       </c>
@@ -994,7 +1001,7 @@
         <v>1234567890</v>
       </c>
     </row>
-    <row r="4" spans="1:27" ht="25" x14ac:dyDescent="0.25">
+    <row ht="25" r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>53</v>
       </c>
@@ -1023,7 +1030,7 @@
         <v>1234567890</v>
       </c>
     </row>
-    <row r="5" spans="1:27" ht="38" customHeight="1" x14ac:dyDescent="0.25">
+    <row customHeight="1" ht="38" r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>53</v>
       </c>
@@ -1076,7 +1083,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:27" ht="37.5" x14ac:dyDescent="0.25">
+    <row ht="37.5" r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>53</v>
       </c>
@@ -1129,7 +1136,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:27" ht="37.5" x14ac:dyDescent="0.25">
+    <row ht="37.5" r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>53</v>
       </c>
@@ -1185,7 +1192,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:27" ht="37.5" x14ac:dyDescent="0.25">
+    <row ht="37.5" r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>53</v>
       </c>
@@ -1217,7 +1224,7 @@
         <v>22201</v>
       </c>
     </row>
-    <row r="9" spans="1:27" ht="37.5" x14ac:dyDescent="0.25">
+    <row ht="37.5" r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>53</v>
       </c>
@@ -1246,7 +1253,7 @@
         <v>22201</v>
       </c>
     </row>
-    <row r="10" spans="1:27" ht="37.5" x14ac:dyDescent="0.25">
+    <row ht="37.5" r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>53</v>
       </c>
@@ -1278,51 +1285,51 @@
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="J2" r:id="rId1" xr:uid="{742F3F73-E85A-4FCF-8C7C-C1600E23D754}"/>
-    <hyperlink ref="J4" r:id="rId2" xr:uid="{CF8BFE12-A940-4AA8-89E5-909545A781DB}"/>
-    <hyperlink ref="J5" r:id="rId3" xr:uid="{C88919CB-0AC0-489E-8BBE-E6060EF3457D}"/>
-    <hyperlink ref="J7" r:id="rId4" xr:uid="{B9848D99-3F02-4B1F-B147-DEC60651F43B}"/>
-    <hyperlink ref="J8" r:id="rId5" xr:uid="{FDA63C53-C5A4-429D-B203-33CB3003E9B2}"/>
-    <hyperlink ref="J9" r:id="rId6" xr:uid="{4707D785-3286-488B-9C77-6EC977F6DD2D}"/>
+    <hyperlink r:id="rId1" ref="J2" xr:uid="{742F3F73-E85A-4FCF-8C7C-C1600E23D754}"/>
+    <hyperlink r:id="rId2" ref="J4" xr:uid="{CF8BFE12-A940-4AA8-89E5-909545A781DB}"/>
+    <hyperlink r:id="rId3" ref="J5" xr:uid="{C88919CB-0AC0-489E-8BBE-E6060EF3457D}"/>
+    <hyperlink r:id="rId4" ref="J7" xr:uid="{B9848D99-3F02-4B1F-B147-DEC60651F43B}"/>
+    <hyperlink r:id="rId5" ref="J8" xr:uid="{FDA63C53-C5A4-429D-B203-33CB3003E9B2}"/>
+    <hyperlink r:id="rId6" ref="J9" xr:uid="{4707D785-3286-488B-9C77-6EC977F6DD2D}"/>
   </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="portrait" r:id="rId7"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35650B67-EEEE-43A0-9B0F-50672085E657}">
-  <dimension ref="A1:AB11"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35650B67-EEEE-43A0-9B0F-50672085E657}">
+  <dimension ref="A1:AC11"/>
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.26953125" style="6" customWidth="1" collapsed="1"/>
-    <col min="2" max="2" width="15.90625" style="6" customWidth="1" collapsed="1"/>
-    <col min="3" max="3" width="36" style="11" customWidth="1" collapsed="1"/>
-    <col min="4" max="4" width="8.7265625" style="6" collapsed="1"/>
-    <col min="5" max="5" width="25.1796875" style="6" bestFit="1" customWidth="1" collapsed="1"/>
-    <col min="6" max="6" width="9.36328125" style="6" customWidth="1" collapsed="1"/>
-    <col min="7" max="7" width="11.36328125" style="6" customWidth="1" collapsed="1"/>
-    <col min="8" max="8" width="10.7265625" style="6" customWidth="1" collapsed="1"/>
-    <col min="9" max="9" width="10.54296875" style="6" customWidth="1" collapsed="1"/>
-    <col min="10" max="10" width="16.453125" style="6" customWidth="1" collapsed="1"/>
-    <col min="11" max="11" width="12" style="6" customWidth="1" collapsed="1"/>
-    <col min="12" max="12" width="16" style="6" customWidth="1" collapsed="1"/>
-    <col min="13" max="13" width="13.26953125" style="6" customWidth="1" collapsed="1"/>
-    <col min="14" max="14" width="13.453125" style="6" customWidth="1" collapsed="1"/>
-    <col min="15" max="16" width="8.7265625" style="6" collapsed="1"/>
-    <col min="17" max="17" width="13.90625" style="6" bestFit="1" customWidth="1" collapsed="1"/>
-    <col min="18" max="18" width="9.54296875" style="6" customWidth="1" collapsed="1"/>
-    <col min="19" max="19" width="10.81640625" style="6" bestFit="1" customWidth="1" collapsed="1"/>
-    <col min="20" max="20" width="8.7265625" style="6" collapsed="1"/>
-    <col min="21" max="21" width="10.26953125" style="6" customWidth="1" collapsed="1"/>
-    <col min="22" max="22" width="6.54296875" style="6" customWidth="1" collapsed="1"/>
-    <col min="23" max="23" width="6.26953125" style="6" customWidth="1" collapsed="1"/>
-    <col min="24" max="24" width="6" style="6" customWidth="1" collapsed="1"/>
-    <col min="25" max="25" width="8.453125" style="6" customWidth="1" collapsed="1"/>
-    <col min="26" max="26" width="5.6328125" style="6" customWidth="1" collapsed="1"/>
-    <col min="27" max="27" width="6.54296875" style="6" customWidth="1" collapsed="1"/>
-    <col min="28" max="28" width="47.08984375" style="11" customWidth="1" collapsed="1"/>
-    <col min="29" max="16384" width="8.7265625" style="6" collapsed="1"/>
+    <col min="1" max="1" customWidth="true" style="6" width="7.26953125" collapsed="true"/>
+    <col min="2" max="2" customWidth="true" style="6" width="15.90625" collapsed="true"/>
+    <col min="3" max="3" customWidth="true" style="11" width="36.0" collapsed="true"/>
+    <col min="4" max="4" style="6" width="8.7265625" collapsed="true"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" style="6" width="25.1796875" collapsed="true"/>
+    <col min="6" max="6" customWidth="true" style="6" width="9.36328125" collapsed="true"/>
+    <col min="7" max="7" customWidth="true" style="6" width="11.36328125" collapsed="true"/>
+    <col min="8" max="8" customWidth="true" style="6" width="10.7265625" collapsed="true"/>
+    <col min="9" max="9" customWidth="true" style="6" width="10.54296875" collapsed="true"/>
+    <col min="10" max="10" customWidth="true" style="6" width="16.453125" collapsed="true"/>
+    <col min="11" max="11" customWidth="true" style="6" width="12.0" collapsed="true"/>
+    <col min="12" max="12" customWidth="true" style="6" width="16.0" collapsed="true"/>
+    <col min="13" max="13" customWidth="true" style="6" width="13.26953125" collapsed="true"/>
+    <col min="14" max="14" customWidth="true" style="6" width="13.453125" collapsed="true"/>
+    <col min="15" max="16" style="6" width="8.7265625" collapsed="true"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" style="6" width="13.90625" collapsed="true"/>
+    <col min="18" max="18" customWidth="true" style="6" width="9.54296875" collapsed="true"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" style="6" width="10.81640625" collapsed="true"/>
+    <col min="20" max="20" style="6" width="8.7265625" collapsed="true"/>
+    <col min="21" max="21" customWidth="true" style="6" width="10.26953125" collapsed="true"/>
+    <col min="22" max="22" customWidth="true" style="6" width="6.54296875" collapsed="true"/>
+    <col min="23" max="23" customWidth="true" style="6" width="6.26953125" collapsed="true"/>
+    <col min="24" max="24" customWidth="true" style="6" width="6.0" collapsed="true"/>
+    <col min="25" max="25" customWidth="true" style="6" width="8.453125" collapsed="true"/>
+    <col min="26" max="26" customWidth="true" style="6" width="5.6328125" collapsed="true"/>
+    <col min="27" max="27" customWidth="true" style="6" width="6.54296875" collapsed="true"/>
+    <col min="28" max="28" customWidth="true" style="11" width="47.08984375" collapsed="true"/>
+    <col min="29" max="16384" style="6" width="8.7265625" collapsed="true"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28" x14ac:dyDescent="0.25">
@@ -1411,12 +1418,12 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="37.5" x14ac:dyDescent="0.25">
+    <row ht="37.5" r="2" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>55</v>
+        <v>85</v>
       </c>
       <c r="C2" s="11" t="s">
         <v>48</v>
@@ -1458,7 +1465,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:28" ht="13" x14ac:dyDescent="0.25">
+    <row ht="13" r="3" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>53</v>
       </c>
@@ -1476,7 +1483,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:28" ht="13" x14ac:dyDescent="0.25">
+    <row ht="13" r="4" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>53</v>
       </c>
@@ -1496,7 +1503,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:28" ht="25" x14ac:dyDescent="0.25">
+    <row ht="25" r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>53</v>
       </c>
@@ -1544,7 +1551,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:28" ht="25" x14ac:dyDescent="0.25">
+    <row ht="25" r="6" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>53</v>
       </c>
@@ -1574,7 +1581,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:28" ht="25" x14ac:dyDescent="0.25">
+    <row ht="25" r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>53</v>
       </c>
@@ -1606,7 +1613,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="8" spans="1:28" ht="25" x14ac:dyDescent="0.25">
+    <row ht="25" r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>53</v>
       </c>
@@ -1638,7 +1645,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="1:28" ht="25" x14ac:dyDescent="0.25">
+    <row ht="25" r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>53</v>
       </c>
@@ -1664,7 +1671,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="10" spans="1:28" ht="25" x14ac:dyDescent="0.25">
+    <row ht="25" r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>53</v>
       </c>
@@ -1754,11 +1761,11 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="J5" r:id="rId1" xr:uid="{588BBDB7-5B95-4FB9-AD9C-36AAC3C41943}"/>
-    <hyperlink ref="J6" r:id="rId2" xr:uid="{CE0F2039-EED1-4DB0-83C0-2B84DB370934}"/>
-    <hyperlink ref="J7" r:id="rId3" xr:uid="{1B3C72AA-06CB-4051-818C-C62CA26213EB}"/>
+    <hyperlink r:id="rId1" ref="J5" xr:uid="{588BBDB7-5B95-4FB9-AD9C-36AAC3C41943}"/>
+    <hyperlink r:id="rId2" ref="J6" xr:uid="{CE0F2039-EED1-4DB0-83C0-2B84DB370934}"/>
+    <hyperlink r:id="rId3" ref="J7" xr:uid="{1B3C72AA-06CB-4051-818C-C62CA26213EB}"/>
   </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>